<commit_message>
MMI order sheet: new header image, columns widen to fit, left-aligned qty, rows match the items
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KhYexLHVfL4ffg26g4b1wU
</commit_message>
<xml_diff>
--- a/src/lib/templates/mmi-order.xlsx
+++ b/src/lib/templates/mmi-order.xlsx
@@ -261,28 +261,17 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:twoCellAnchor editAs="oneCell">
+  <xdr:oneCellAnchor>
     <xdr:from>
       <xdr:col>2</xdr:col>
       <xdr:colOff>0</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2295845</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>495369</xdr:rowOff>
-    </xdr:to>
+    <xdr:ext cx="5219700" cy="457200"/>
     <xdr:pic>
       <xdr:nvPicPr>
-        <xdr:cNvPr id="2" name="Picture 1">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{DDEC79F5-8E26-95E5-BADD-545F281D03F8}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
+        <xdr:cNvPr id="2" name="POSM SHOP header" descr="Sirocco POSM SHOP - New order"/>
         <xdr:cNvPicPr>
           <a:picLocks noChangeAspect="1"/>
         </xdr:cNvPicPr>
@@ -296,7 +285,7 @@
       <xdr:spPr>
         <a:xfrm>
           <a:off x="0" y="0"/>
-          <a:ext cx="2295845" cy="495369"/>
+          <a:ext cx="5219700" cy="457200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -304,123 +293,7 @@
       </xdr:spPr>
     </xdr:pic>
     <xdr:clientData/>
-  </xdr:twoCellAnchor>
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2432539</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>109905</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1104854" cy="311496"/>
-    <xdr:sp macro="" textlink="">
-      <xdr:nvSpPr>
-        <xdr:cNvPr id="3" name="TextBox 2">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CA4E1B08-975D-2993-AE1F-3F0197B0389A}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvSpPr txBox="1"/>
-      </xdr:nvSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3135924" y="183174"/>
-          <a:ext cx="1104854" cy="311496"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:fillRef>
-        <a:effectRef idx="0">
-          <a:scrgbClr r="0" g="0" b="0"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-      <xdr:txBody>
-        <a:bodyPr vertOverflow="clip" horzOverflow="clip" wrap="none" rtlCol="0" anchor="t">
-          <a:spAutoFit/>
-        </a:bodyPr>
-        <a:lstStyle/>
-        <a:p>
-          <a:r>
-            <a:rPr lang="en-GB" sz="1400" b="1"/>
-            <a:t>NEW ORDER</a:t>
-          </a:r>
-          <a:endParaRPr lang="en-GB" sz="1100" b="1"/>
-        </a:p>
-      </xdr:txBody>
-    </xdr:sp>
-    <xdr:clientData/>
   </xdr:oneCellAnchor>
-  <xdr:twoCellAnchor>
-    <xdr:from>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2351942</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>87923</xdr:rowOff>
-    </xdr:from>
-    <xdr:to>
-      <xdr:col>2</xdr:col>
-      <xdr:colOff>2351942</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>373673</xdr:rowOff>
-    </xdr:to>
-    <xdr:cxnSp macro="">
-      <xdr:nvCxnSpPr>
-        <xdr:cNvPr id="5" name="Straight Connector 4">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{AA78C730-2228-A06F-76B5-4904AB29FA93}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvCxnSpPr/>
-      </xdr:nvCxnSpPr>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="3055327" y="161192"/>
-          <a:ext cx="0" cy="285750"/>
-        </a:xfrm>
-        <a:prstGeom prst="line">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:ln w="9525">
-          <a:solidFill>
-            <a:schemeClr val="bg1">
-              <a:lumMod val="85000"/>
-            </a:schemeClr>
-          </a:solidFill>
-        </a:ln>
-      </xdr:spPr>
-      <xdr:style>
-        <a:lnRef idx="2">
-          <a:schemeClr val="accent1"/>
-        </a:lnRef>
-        <a:fillRef idx="0">
-          <a:schemeClr val="accent1"/>
-        </a:fillRef>
-        <a:effectRef idx="1">
-          <a:schemeClr val="accent1"/>
-        </a:effectRef>
-        <a:fontRef idx="minor">
-          <a:schemeClr val="tx1"/>
-        </a:fontRef>
-      </xdr:style>
-    </xdr:cxnSp>
-    <xdr:clientData/>
-  </xdr:twoCellAnchor>
 </xdr:wsDr>
 </file>
 

</xml_diff>